<commit_message>
docs: complete Templates 0, 2, 3 and remove unused files in folder_template
</commit_message>
<xml_diff>
--- a/folder_template/Template0_AI Usage Report.xlsx
+++ b/folder_template/Template0_AI Usage Report.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11880"/>
+    <workbookView windowWidth="19200" windowHeight="8000" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="0.Overview" sheetId="1" r:id="rId1"/>
@@ -1498,12 +1498,12 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="12.6666666666667" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="12.6636363636364" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="21.3333333333333" style="1" customWidth="1"/>
-    <col min="2" max="2" width="32.8857142857143" customWidth="1"/>
-    <col min="3" max="3" width="30.2190476190476" customWidth="1"/>
-    <col min="5" max="5" width="32.552380952381" customWidth="1"/>
+    <col min="1" max="1" width="21.3363636363636" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32.8818181818182" customWidth="1"/>
+    <col min="3" max="3" width="30.2181818181818" customWidth="1"/>
+    <col min="5" max="5" width="32.5545454545455" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1" spans="1:5">
@@ -1592,7 +1592,7 @@
       <c r="D8" s="21"/>
       <c r="E8" s="21"/>
     </row>
-    <row r="9" ht="12.75" spans="1:5">
+    <row r="9" ht="12.5" spans="1:5">
       <c r="B9" s="22"/>
     </row>
     <row r="10" ht="13" customHeight="1" spans="1:5">
@@ -1621,7 +1621,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" ht="12.5" spans="1:5">
       <c r="A12" s="23">
         <v>1</v>
       </c>
@@ -1638,7 +1638,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" ht="12.75" spans="1:5">
+    <row r="13" ht="12.5" spans="1:5">
       <c r="A13" s="23">
         <v>2</v>
       </c>
@@ -1655,7 +1655,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" ht="12.75" spans="1:5">
+    <row r="14" ht="12.5" spans="1:5">
       <c r="A14" s="23">
         <v>3</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" ht="12.75" spans="1:5">
+    <row r="15" ht="12.5" spans="1:5">
       <c r="A15" s="23">
         <v>4</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" ht="12.75" spans="1:5">
+    <row r="16" ht="12.5" spans="1:5">
       <c r="A16" s="23">
         <v>5</v>
       </c>
@@ -1722,17 +1722,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Y7"/>
-  <sheetFormatPr defaultColWidth="12.6666666666667" defaultRowHeight="12.75" outlineLevelRow="6"/>
+  <sheetFormatPr defaultColWidth="12.6636363636364" defaultRowHeight="12.5" outlineLevelRow="6"/>
   <cols>
-    <col min="1" max="1" width="9.21904761904762" customWidth="1"/>
-    <col min="2" max="2" width="18.8857142857143" customWidth="1"/>
-    <col min="3" max="3" width="18.552380952381" customWidth="1"/>
-    <col min="5" max="5" width="20.6666666666667" customWidth="1"/>
-    <col min="6" max="6" width="23.2190476190476" customWidth="1"/>
+    <col min="1" max="1" width="9.21818181818182" customWidth="1"/>
+    <col min="2" max="2" width="18.8818181818182" customWidth="1"/>
+    <col min="3" max="3" width="18.5545454545455" customWidth="1"/>
+    <col min="5" max="5" width="20.6636363636364" customWidth="1"/>
+    <col min="6" max="6" width="23.2181818181818" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="15.8857142857143" customWidth="1"/>
-    <col min="9" max="9" width="13.447619047619" customWidth="1"/>
-    <col min="10" max="10" width="25.552380952381" customWidth="1"/>
+    <col min="8" max="8" width="15.8818181818182" customWidth="1"/>
+    <col min="9" max="9" width="13.4454545454545" customWidth="1"/>
+    <col min="10" max="10" width="25.5545454545455" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:25">
@@ -1940,7 +1940,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" ht="89.25" spans="1:25">
+    <row r="6" ht="87.5" spans="1:25">
       <c r="A6" s="11" t="s">
         <v>71</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="7" ht="89.25" spans="1:25">
+    <row r="7" ht="87.5" spans="1:25">
       <c r="A7" s="11" t="s">
         <v>79</v>
       </c>
@@ -2016,19 +2016,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Y9"/>
-  <sheetFormatPr defaultColWidth="12.6666666666667" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="12.6636363636364" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="10.1142857142857" style="9" customWidth="1"/>
-    <col min="2" max="2" width="22.8857142857143" style="9" customWidth="1"/>
+    <col min="1" max="1" width="10.1181818181818" style="9" customWidth="1"/>
+    <col min="2" max="2" width="22.8818181818182" style="9" customWidth="1"/>
     <col min="3" max="3" width="19" style="9" customWidth="1"/>
-    <col min="4" max="4" width="12.6666666666667" style="9" customWidth="1"/>
-    <col min="5" max="5" width="20.6666666666667" style="9" customWidth="1"/>
-    <col min="6" max="6" width="25.3333333333333" style="9" customWidth="1"/>
-    <col min="7" max="7" width="16.552380952381" style="9" customWidth="1"/>
-    <col min="8" max="8" width="24.3333333333333" style="9" customWidth="1"/>
-    <col min="9" max="9" width="13.2190476190476" style="9" customWidth="1"/>
-    <col min="10" max="10" width="29.447619047619" style="9" customWidth="1"/>
-    <col min="11" max="16384" width="12.6666666666667" style="9" customWidth="1"/>
+    <col min="4" max="4" width="12.6636363636364" style="9" customWidth="1"/>
+    <col min="5" max="5" width="20.6636363636364" style="9" customWidth="1"/>
+    <col min="6" max="6" width="25.3363636363636" style="9" customWidth="1"/>
+    <col min="7" max="7" width="16.5545454545455" style="9" customWidth="1"/>
+    <col min="8" max="8" width="24.3363636363636" style="9" customWidth="1"/>
+    <col min="9" max="9" width="13.2181818181818" style="9" customWidth="1"/>
+    <col min="10" max="10" width="29.4454545454545" style="9" customWidth="1"/>
+    <col min="11" max="16384" width="12.6636363636364" style="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:25">
@@ -2154,7 +2154,7 @@
       <c r="O3" s="12"/>
       <c r="P3" s="12"/>
     </row>
-    <row r="4" ht="114.75" spans="1:25">
+    <row r="4" ht="112.5" spans="1:25">
       <c r="A4" s="11" t="s">
         <v>102</v>
       </c>
@@ -2186,7 +2186,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="5" ht="63.75" spans="1:25">
+    <row r="5" ht="50" spans="1:25">
       <c r="A5" s="11" t="s">
         <v>93</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" ht="89.25" spans="1:25">
+    <row r="6" ht="75" spans="1:25">
       <c r="A6" s="13" t="s">
         <v>71</v>
       </c>
@@ -2250,7 +2250,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" ht="102" spans="1:25">
+    <row r="7" ht="87.5" spans="1:25">
       <c r="A7" s="13" t="s">
         <v>79</v>
       </c>
@@ -2282,7 +2282,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" ht="114.75" spans="1:25">
+    <row r="8" ht="87.5" spans="1:25">
       <c r="A8" s="13" t="s">
         <v>125</v>
       </c>
@@ -2314,7 +2314,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="9" ht="89.25" spans="1:25">
+    <row r="9" ht="87.5" spans="1:25">
       <c r="A9" s="13" t="s">
         <v>131</v>
       </c>
@@ -2358,9 +2358,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="12.6666666666667" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="12.6636363636364" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="27.1142857142857" style="1" customWidth="1"/>
+    <col min="1" max="1" width="27.1181818181818" style="1" customWidth="1"/>
     <col min="2" max="2" width="93" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>